<commit_message>
Committing Generated Files 7
</commit_message>
<xml_diff>
--- a/manual_tests/login_approved_manual_tests.xlsx
+++ b/manual_tests/login_approved_manual_tests.xlsx
@@ -508,14 +508,14 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Open a web browser
+          <t>Open a browser
 Navigate to http://172.21.166.115/washtabui/login?data=undefined
 Observe the login page UI</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Login page loads successfully and displays login form elements including username field, password field, and login button.</t>
+          <t>Login page loads successfully and displays login form elements such as username field, password field, and login button.</t>
         </is>
       </c>
     </row>
@@ -561,14 +561,14 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>User is authenticated successfully and redirected to the application home or dashboard page.</t>
+          <t>User is successfully authenticated and redirected to the application landing page.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AUT-LOGIN03: Verify login fails with incorrect username</t>
+          <t>AUT-LOGIN03: Verify login failure with incorrect username and valid password</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -583,7 +583,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Verify login fails with incorrect username</t>
+          <t>Verify login failure with incorrect username and valid password</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -600,21 +600,21 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>Open the login page
-Enter username invaliduser in the username field
-Enter password Icstunnel1 in the password field
+Enter an incorrect username such as wronguser
+Enter password Icstunnel1
 Click the Login button</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Login attempt fails and an error message indicating invalid username or password is displayed.</t>
+          <t>Login fails and an error message indicating invalid username or password is displayed.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AUT-LOGIN04: Verify login fails with incorrect password</t>
+          <t>AUT-LOGIN04: Verify login failure with valid username and incorrect password</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Verify login fails with incorrect password</t>
+          <t>Verify login failure with valid username and incorrect password</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -646,21 +646,21 @@
       <c r="H5" t="inlineStr">
         <is>
           <t>Open the login page
-Enter username haklarr in the username field
-Enter password WrongPassword in the password field
+Enter username haklarr
+Enter an incorrect password such as WrongPass123
 Click the Login button</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Login attempt fails and an error message indicating invalid username or password is displayed.</t>
+          <t>Login fails and an error message indicating invalid username or password is displayed.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AUT-LOGIN05: Verify login fails when both username and password are blank</t>
+          <t>AUT-LOGIN05: Verify login failure when both username and password are blank</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Verify login fails when both username and password are blank</t>
+          <t>Verify login failure when both username and password are blank</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -692,21 +692,21 @@
       <c r="H6" t="inlineStr">
         <is>
           <t>Open the login page
-Leave username field blank
-Leave password field blank
+Leave username field empty
+Leave password field empty
 Click the Login button</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Login is rejected and validation or error message indicates that username and password cannot be blank.</t>
+          <t>Login fails and a validation or error message is displayed indicating credentials are required.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AUT-LOGIN06: Verify login fails when username is blank</t>
+          <t>AUT-LOGIN06: Verify login failure when username is blank</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Verify login fails when username is blank</t>
+          <t>Verify login failure when username is blank</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -738,21 +738,21 @@
       <c r="H7" t="inlineStr">
         <is>
           <t>Open the login page
-Leave username field blank
+Leave the username field empty
 Enter password Icstunnel1
 Click the Login button</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Login is rejected and validation message indicates username is required.</t>
+          <t>Login fails and an error message is displayed indicating invalid username or password or missing username.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AUT-LOGIN07: Verify login fails when password is blank</t>
+          <t>AUT-LOGIN07: Verify login failure when password is blank</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -767,7 +767,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Verify login fails when password is blank</t>
+          <t>Verify login failure when password is blank</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -785,20 +785,20 @@
         <is>
           <t>Open the login page
 Enter username haklarr
-Leave password field blank
+Leave the password field empty
 Click the Login button</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Login is rejected and validation message indicates password is required.</t>
+          <t>Login fails and an error message is displayed indicating invalid username or password or missing password.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AUT-LOGIN08: Verify username field accepts leading and trailing spaces</t>
+          <t>AUT-LOGIN08: Verify login with leading and trailing spaces in username</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Verify username field accepts leading and trailing spaces</t>
+          <t>Verify login with leading and trailing spaces in username</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -830,21 +830,21 @@
       <c r="H9" t="inlineStr">
         <is>
           <t>Open the login page
-Enter username with spaces before and after value such as space haklarr space
+Enter username with spaces such as '  haklarr  '
 Enter password Icstunnel1
 Click the Login button</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>System trims leading and trailing spaces or rejects the login attempt with appropriate validation.</t>
+          <t>System either trims whitespace and logs the user in successfully or rejects the login with an appropriate validation message.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AUT-LOGIN09: Verify password field accepts leading and trailing spaces</t>
+          <t>AUT-LOGIN09: Verify login with leading and trailing spaces in password</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Verify password field accepts leading and trailing spaces</t>
+          <t>Verify login with leading and trailing spaces in password</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -877,20 +877,20 @@
         <is>
           <t>Open the login page
 Enter username haklarr
-Enter password with leading and trailing spaces around Icstunnel1
+Enter password with spaces such as '  Icstunnel1  '
 Click the Login button</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>System handles leading and trailing spaces appropriately and either trims them or rejects login with a validation message.</t>
+          <t>Authentication should follow system password rules and either trim spaces or reject login with an error message.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AUT-LOGIN10: Verify login fails with whitespace-only username and password</t>
+          <t>AUT-LOGIN10: Verify login failure with special characters in username</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Verify login fails with whitespace-only username and password</t>
+          <t>Verify login failure with special characters in username</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -922,21 +922,21 @@
       <c r="H11" t="inlineStr">
         <is>
           <t>Open the login page
-Enter spaces only in username field
-Enter spaces only in password field
+Enter username such as haklarr!@#
+Enter password Icstunnel1
 Click the Login button</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Login is rejected and validation indicates fields cannot contain only whitespace.</t>
+          <t>Login fails and appropriate validation or authentication error is displayed.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AUT-LOGIN11: Verify login fails with very long username input</t>
+          <t>AUT-LOGIN11: Verify login failure with SQL injection style input</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -951,12 +951,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Verify login fails with very long username input</t>
+          <t>Verify login failure with SQL injection style input</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -968,21 +968,21 @@
       <c r="H12" t="inlineStr">
         <is>
           <t>Open the login page
-Enter a very long string of characters exceeding normal username length in username field
-Enter password Icstunnel1
+Enter username value ' OR '1'='1
+Enter password value ' OR '1'='1
 Click the Login button</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>System handles long input safely and either rejects with validation or processes without breaking the UI.</t>
+          <t>Login attempt is rejected and the system does not authenticate the user.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AUT-LOGIN12: Verify login fails with very long password input</t>
+          <t>AUT-LOGIN12: Verify login failure with extremely long username input</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -997,7 +997,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Verify login fails with very long password input</t>
+          <t>Verify login failure with extremely long username input</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1014,21 +1014,21 @@
       <c r="H13" t="inlineStr">
         <is>
           <t>Open the login page
-Enter username haklarr
-Enter an extremely long password string
+Enter a username longer than typical limits such as 256 characters
+Enter password Icstunnel1
 Click the Login button</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>System handles long password input safely without UI or server errors and login fails with appropriate message.</t>
+          <t>System handles the long input gracefully and shows validation or login failure without UI breakage.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AUT-LOGIN13: Verify username field accepts special characters input</t>
+          <t>AUT-LOGIN13: Verify login failure with extremely long password input</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Verify username field accepts special characters input</t>
+          <t>Verify login failure with extremely long password input</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1060,21 +1060,21 @@
       <c r="H14" t="inlineStr">
         <is>
           <t>Open the login page
-Enter username containing special characters such as user!@#
-Enter password Icstunnel1
+Enter username haklarr
+Enter a password longer than typical limits such as 256 characters
 Click the Login button</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Login fails and application handles special characters safely without system errors.</t>
+          <t>System handles the long password input gracefully and login fails with an appropriate error message.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AUT-LOGIN14: Verify password field masks entered characters</t>
+          <t>AUT-LOGIN14: Verify username field accepts copy paste input</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Verify password field masks entered characters</t>
+          <t>Verify username field accepts copy paste input</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1106,20 +1106,22 @@
       <c r="H15" t="inlineStr">
         <is>
           <t>Open the login page
-Enter text in the password field
-Observe the characters displayed in the field</t>
+Copy the value haklarr from an external source
+Paste it into the username field
+Enter password Icstunnel1
+Click the Login button</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Password characters are masked and not visible in plain text.</t>
+          <t>Username paste operation works and login succeeds with valid credentials.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AUT-LOGIN15: Verify login using Enter key submission</t>
+          <t>AUT-LOGIN15: Verify password field accepts copy paste input</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1134,12 +1136,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Verify login using Enter key submission</t>
+          <t>Verify password field accepts copy paste input</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1152,20 +1154,21 @@
         <is>
           <t>Open the login page
 Enter username haklarr
-Enter password Icstunnel1
-Press Enter key on keyboard</t>
+Copy password Icstunnel1
+Paste it into the password field
+Click the Login button</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Login form is submitted and user is logged in successfully.</t>
+          <t>Password paste operation works and login succeeds with valid credentials.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AUT-LOGIN16: Verify login fails with case-sensitive username variation</t>
+          <t>AUT-LOGIN16: Verify login attempt with username in different case</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1180,7 +1183,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Verify login fails with case-sensitive username variation</t>
+          <t>Verify login attempt with username in different case</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1199,19 +1202,19 @@
           <t>Open the login page
 Enter username HAKLARR
 Enter password Icstunnel1
-Click Login</t>
+Click the Login button</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>System processes according to username case-sensitivity rules and either authenticates correctly or shows invalid credentials message.</t>
+          <t>Authentication behavior follows system case sensitivity rules and login either succeeds or fails accordingly.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AUT-LOGIN17: Verify login fails with case-sensitive password variation</t>
+          <t>AUT-LOGIN17: Verify password field masks entered characters</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1226,12 +1229,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Verify login fails with case-sensitive password variation</t>
+          <t>Verify password field masks entered characters</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1243,21 +1246,20 @@
       <c r="H18" t="inlineStr">
         <is>
           <t>Open the login page
-Enter username haklarr
-Enter password icstunnel1
-Click Login</t>
+Click the password field
+Type password Icstunnel1</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Login fails and invalid username or password message is displayed.</t>
+          <t>Password characters are masked or hidden while typing.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AUT-LOGIN18: Verify multiple rapid login button clicks handling</t>
+          <t>AUT-LOGIN18: Verify pressing Enter key submits login form</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1272,7 +1274,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Verify multiple rapid login button clicks handling</t>
+          <t>Verify pressing Enter key submits login form</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1287,6 +1289,52 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
+        <is>
+          <t>Open the login page
+Enter username haklarr
+Enter password Icstunnel1
+Press the Enter key on the keyboard</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Login form is submitted and the user is authenticated successfully.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AUT-LOGIN19: Verify multiple rapid clicks on login button</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>AU-LOGIN19</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>LOGIN_TC_019</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Verify multiple rapid clicks on login button</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
         <is>
           <t>Open the login page
 Enter username haklarr
@@ -1294,63 +1342,16 @@
 Click the Login button multiple times rapidly</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>System processes a single authentication request and prevents duplicate submissions or errors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>AUT-LOGIN19: Verify copy paste functionality for username and password fields</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>AU-LOGIN19</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>LOGIN_TC_019</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Verify copy paste functionality for username and password fields</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Copy username haklarr from an external source
-Paste the value into the username field
-Copy password Icstunnel1 from an external source
-Paste the value into the password field
-Click Login</t>
-        </is>
-      </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Login works correctly using pasted values and user is authenticated successfully.</t>
+          <t>System processes the login request safely and does not create duplicate sessions or UI errors.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AUT-LOGIN20: Verify error message visibility after failed login attempt</t>
+          <t>AUT-LOGIN20: Verify login error message appears after failed login</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1365,7 +1366,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Verify error message visibility after failed login attempt</t>
+          <t>Verify login error message appears after failed login</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1382,14 +1383,14 @@
       <c r="H21" t="inlineStr">
         <is>
           <t>Open the login page
-Enter username wronguser
-Enter password wrongpassword
-Click Login</t>
+Enter username invaliduser
+Enter password invalidpass
+Click the Login button</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>An error message clearly indicating login failure is displayed on the login page.</t>
+          <t>A visible error message is displayed indicating login failure.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Committing Generated Files 8
</commit_message>
<xml_diff>
--- a/manual_tests/login_approved_manual_tests.xlsx
+++ b/manual_tests/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -477,22 +477,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AUT-LOGIN01: Verify login page loads successfully</t>
+          <t>AUT-LOGIN01: Verify login with valid username and password</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AU-LOGIN01</t>
+          <t>WT-LOGIN01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>LOGIN_TC_001</t>
+          <t>TC_LOGIN_001</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Verify login page loads successfully</t>
+          <t>Verify login with valid username and password</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -508,41 +508,42 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Open a browser
-Navigate to http://172.21.166.115/washtabui/login?data=undefined
-Observe the login page UI</t>
+          <t>Open the login page URL in a browser
+Enter username haklarr in the username field
+Enter password Icstunnel1 in the password field
+Click the Login button</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Login page loads successfully and displays login form elements such as username field, password field, and login button.</t>
+          <t>User is successfully authenticated and redirected to the application home/dashboard page.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AUT-LOGIN02: Verify successful login with valid username and password</t>
+          <t>AUT-LOGIN02: Verify login failure with incorrect username and valid password</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AU-LOGIN02</t>
+          <t>WT-LOGIN02</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>LOGIN_TC_002</t>
+          <t>TC_LOGIN_002</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Verify successful login with valid username and password</t>
+          <t>Verify login failure with incorrect username and valid password</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -554,36 +555,36 @@
       <c r="H3" t="inlineStr">
         <is>
           <t>Open the login page
-Enter username haklarr in the username field
-Enter password Icstunnel1 in the password field
+Enter invalid username wronguser
+Enter password Icstunnel1
 Click the Login button</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>User is successfully authenticated and redirected to the application landing page.</t>
+          <t>Login fails and an error message indicating incorrect username or password is displayed.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AUT-LOGIN03: Verify login failure with incorrect username and valid password</t>
+          <t>AUT-LOGIN03: Verify login failure with valid username and incorrect password</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AU-LOGIN03</t>
+          <t>WT-LOGIN03</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LOGIN_TC_003</t>
+          <t>TC_LOGIN_003</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Verify login failure with incorrect username and valid password</t>
+          <t>Verify login failure with valid username and incorrect password</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -600,36 +601,36 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>Open the login page
-Enter an incorrect username such as wronguser
-Enter password Icstunnel1
+Enter username haklarr
+Enter incorrect password wrongpass
 Click the Login button</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Login fails and an error message indicating invalid username or password is displayed.</t>
+          <t>Login fails and an error message indicating incorrect username or password is displayed.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AUT-LOGIN04: Verify login failure with valid username and incorrect password</t>
+          <t>AUT-LOGIN04: Verify login failure when both username and password are incorrect</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AU-LOGIN04</t>
+          <t>WT-LOGIN04</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>LOGIN_TC_004</t>
+          <t>TC_LOGIN_004</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Verify login failure with valid username and incorrect password</t>
+          <t>Verify login failure when both username and password are incorrect</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -646,36 +647,36 @@
       <c r="H5" t="inlineStr">
         <is>
           <t>Open the login page
-Enter username haklarr
-Enter an incorrect password such as WrongPass123
+Enter username invaliduser
+Enter password invalidpass
 Click the Login button</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Login fails and an error message indicating invalid username or password is displayed.</t>
+          <t>Login fails and an error message indicating incorrect username or password is displayed.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AUT-LOGIN05: Verify login failure when both username and password are blank</t>
+          <t>AUT-LOGIN05: Verify validation when username and password fields are blank</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AU-LOGIN05</t>
+          <t>WT-LOGIN05</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LOGIN_TC_005</t>
+          <t>TC_LOGIN_005</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Verify login failure when both username and password are blank</t>
+          <t>Verify validation when username and password fields are blank</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -692,36 +693,36 @@
       <c r="H6" t="inlineStr">
         <is>
           <t>Open the login page
-Leave username field empty
-Leave password field empty
+Leave the username field empty
+Leave the password field empty
 Click the Login button</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Login fails and a validation or error message is displayed indicating credentials are required.</t>
+          <t>Login fails and validation message appears indicating username and password are required.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AUT-LOGIN06: Verify login failure when username is blank</t>
+          <t>AUT-LOGIN06: Verify validation when username is blank and password is entered</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AU-LOGIN06</t>
+          <t>WT-LOGIN06</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>LOGIN_TC_006</t>
+          <t>TC_LOGIN_006</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Verify login failure when username is blank</t>
+          <t>Verify validation when username is blank and password is entered</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -738,36 +739,36 @@
       <c r="H7" t="inlineStr">
         <is>
           <t>Open the login page
-Leave the username field empty
+Leave username field empty
 Enter password Icstunnel1
 Click the Login button</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Login fails and an error message is displayed indicating invalid username or password or missing username.</t>
+          <t>Validation message appears indicating username is required and login is not allowed.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AUT-LOGIN07: Verify login failure when password is blank</t>
+          <t>AUT-LOGIN07: Verify validation when password is blank and username is entered</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AU-LOGIN07</t>
+          <t>WT-LOGIN07</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>LOGIN_TC_007</t>
+          <t>TC_LOGIN_007</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Verify login failure when password is blank</t>
+          <t>Verify validation when password is blank and username is entered</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -785,35 +786,35 @@
         <is>
           <t>Open the login page
 Enter username haklarr
-Leave the password field empty
+Leave password field empty
 Click the Login button</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Login fails and an error message is displayed indicating invalid username or password or missing password.</t>
+          <t>Validation message appears indicating password is required and login is not allowed.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AUT-LOGIN08: Verify login with leading and trailing spaces in username</t>
+          <t>AUT-LOGIN08: Verify username field accepts leading and trailing spaces</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AU-LOGIN08</t>
+          <t>WT-LOGIN08</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LOGIN_TC_008</t>
+          <t>TC_LOGIN_008</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Verify login with leading and trailing spaces in username</t>
+          <t>Verify username field accepts leading and trailing spaces</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -830,36 +831,36 @@
       <c r="H9" t="inlineStr">
         <is>
           <t>Open the login page
-Enter username with spaces such as '  haklarr  '
+Enter username with spaces '  haklarr  '
 Enter password Icstunnel1
 Click the Login button</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>System either trims whitespace and logs the user in successfully or rejects the login with an appropriate validation message.</t>
+          <t>System trims whitespace and authenticates the user successfully if credentials are valid.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AUT-LOGIN09: Verify login with leading and trailing spaces in password</t>
+          <t>AUT-LOGIN09: Verify password field with leading and trailing spaces</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AU-LOGIN09</t>
+          <t>WT-LOGIN09</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>LOGIN_TC_009</t>
+          <t>TC_LOGIN_009</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Verify login with leading and trailing spaces in password</t>
+          <t>Verify password field with leading and trailing spaces</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -877,35 +878,35 @@
         <is>
           <t>Open the login page
 Enter username haklarr
-Enter password with spaces such as '  Icstunnel1  '
+Enter password with spaces '  Icstunnel1  '
 Click the Login button</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Authentication should follow system password rules and either trim spaces or reject login with an error message.</t>
+          <t>Login fails if spaces are treated as characters or succeeds if spaces are trimmed based on system behavior.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AUT-LOGIN10: Verify login failure with special characters in username</t>
+          <t>AUT-LOGIN10: Verify login attempt using only whitespace characters</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>AU-LOGIN10</t>
+          <t>WT-LOGIN10</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>LOGIN_TC_010</t>
+          <t>TC_LOGIN_010</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Verify login failure with special characters in username</t>
+          <t>Verify login attempt using only whitespace characters</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -922,41 +923,41 @@
       <c r="H11" t="inlineStr">
         <is>
           <t>Open the login page
-Enter username such as haklarr!@#
-Enter password Icstunnel1
+Enter spaces in username field
+Enter spaces in password field
 Click the Login button</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Login fails and appropriate validation or authentication error is displayed.</t>
+          <t>Validation error appears indicating username and password cannot be blank or whitespace.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AUT-LOGIN11: Verify login failure with SQL injection style input</t>
+          <t>AUT-LOGIN11: Verify login with very long username input</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AU-LOGIN11</t>
+          <t>WT-LOGIN11</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>LOGIN_TC_011</t>
+          <t>TC_LOGIN_011</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Verify login failure with SQL injection style input</t>
+          <t>Verify login with very long username input</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -968,36 +969,36 @@
       <c r="H12" t="inlineStr">
         <is>
           <t>Open the login page
-Enter username value ' OR '1'='1
-Enter password value ' OR '1'='1
+Enter a very long username string exceeding typical length limits
+Enter password Icstunnel1
 Click the Login button</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Login attempt is rejected and the system does not authenticate the user.</t>
+          <t>System prevents excessive input or displays validation without crashing or breaking UI.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AUT-LOGIN12: Verify login failure with extremely long username input</t>
+          <t>AUT-LOGIN12: Verify login with very long password input</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>AU-LOGIN12</t>
+          <t>WT-LOGIN12</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>LOGIN_TC_012</t>
+          <t>TC_LOGIN_012</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Verify login failure with extremely long username input</t>
+          <t>Verify login with very long password input</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1014,36 +1015,36 @@
       <c r="H13" t="inlineStr">
         <is>
           <t>Open the login page
-Enter a username longer than typical limits such as 256 characters
-Enter password Icstunnel1
+Enter username haklarr
+Enter a very long password string exceeding typical limits
 Click the Login button</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>System handles the long input gracefully and shows validation or login failure without UI breakage.</t>
+          <t>System handles long password input safely and shows appropriate login failure or validation.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AUT-LOGIN13: Verify login failure with extremely long password input</t>
+          <t>AUT-LOGIN13: Verify login with special characters in username</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>AU-LOGIN13</t>
+          <t>WT-LOGIN13</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>LOGIN_TC_013</t>
+          <t>TC_LOGIN_013</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Verify login failure with extremely long password input</t>
+          <t>Verify login with special characters in username</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1060,36 +1061,36 @@
       <c r="H14" t="inlineStr">
         <is>
           <t>Open the login page
-Enter username haklarr
-Enter a password longer than typical limits such as 256 characters
+Enter username haklarr!@#
+Enter password Icstunnel1
 Click the Login button</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>System handles the long password input gracefully and login fails with an appropriate error message.</t>
+          <t>Login fails gracefully and system handles special characters without UI errors.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AUT-LOGIN14: Verify username field accepts copy paste input</t>
+          <t>AUT-LOGIN14: Verify login with special characters in password</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>AU-LOGIN14</t>
+          <t>WT-LOGIN14</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>LOGIN_TC_014</t>
+          <t>TC_LOGIN_014</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Verify username field accepts copy paste input</t>
+          <t>Verify login with special characters in password</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1106,42 +1107,41 @@
       <c r="H15" t="inlineStr">
         <is>
           <t>Open the login page
-Copy the value haklarr from an external source
-Paste it into the username field
-Enter password Icstunnel1
+Enter username haklarr
+Enter password Icstunnel1!@#
 Click the Login button</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Username paste operation works and login succeeds with valid credentials.</t>
+          <t>System processes input normally and login fails unless the password exactly matches stored credentials.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AUT-LOGIN15: Verify password field accepts copy paste input</t>
+          <t>AUT-LOGIN15: Verify login button is visible on login page</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>AU-LOGIN15</t>
+          <t>WT-LOGIN15</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>LOGIN_TC_015</t>
+          <t>TC_LOGIN_015</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Verify password field accepts copy paste input</t>
+          <t>Verify login button is visible on login page</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1153,42 +1153,39 @@
       <c r="H16" t="inlineStr">
         <is>
           <t>Open the login page
-Enter username haklarr
-Copy password Icstunnel1
-Paste it into the password field
-Click the Login button</t>
+Observe the login form UI</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Password paste operation works and login succeeds with valid credentials.</t>
+          <t>Username field, password field, and Login button are visible and properly aligned on the page.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AUT-LOGIN16: Verify login attempt with username in different case</t>
+          <t>AUT-LOGIN16: Verify password field masks entered characters</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>AU-LOGIN16</t>
+          <t>WT-LOGIN16</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>LOGIN_TC_016</t>
+          <t>TC_LOGIN_016</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Verify login attempt with username in different case</t>
+          <t>Verify password field masks entered characters</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1200,197 +1197,287 @@
       <c r="H17" t="inlineStr">
         <is>
           <t>Open the login page
+Click on the password field
+Enter any password characters</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Entered password characters are masked or hidden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>AUT-LOGIN17: Verify pressing Enter key submits login form</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>WT-LOGIN17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_017</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Verify pressing Enter key submits login form</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Open the login page
+Enter username haklarr
+Enter password Icstunnel1
+Press the Enter key on keyboard</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Login form submits and user is logged in successfully.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>AUT-LOGIN18: Verify multiple rapid clicks on login button</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>WT-LOGIN18</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_018</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Verify multiple rapid clicks on login button</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Open the login page
+Enter username haklarr
+Enter password Icstunnel1
+Rapidly click the Login button multiple times</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>System processes login once and prevents duplicate submissions or errors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AUT-LOGIN19: Verify copy paste of credentials into fields</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>WT-LOGIN19</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_019</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Verify copy paste of credentials into fields</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Open the login page
+Copy username haklarr and paste into username field
+Copy password Icstunnel1 and paste into password field
+Click the Login button</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Login succeeds and user is redirected to the dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>AUT-LOGIN20: Verify case sensitivity of username</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>WT-LOGIN20</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_020</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Verify case sensitivity of username</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Open the login page
 Enter username HAKLARR
 Enter password Icstunnel1
 Click the Login button</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Authentication behavior follows system case sensitivity rules and login either succeeds or fails accordingly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>AUT-LOGIN17: Verify password field masks entered characters</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>AU-LOGIN17</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>LOGIN_TC_017</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Verify password field masks entered characters</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Login succeeds or fails based on system case sensitivity rules but does not break authentication flow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>AUT-LOGIN21: Verify case sensitivity of password</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>WT-LOGIN21</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_021</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Verify case sensitivity of password</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Open the login page
+Enter username haklarr
+Enter password icstunnel1
+Click the Login button</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Login fails because password case does not match.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>AUT-LOGIN22: Verify login page loads successfully</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>WT-LOGIN22</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_022</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Verify login page loads successfully</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Open the login page
-Click the password field
-Type password Icstunnel1</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Password characters are masked or hidden while typing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>AUT-LOGIN18: Verify pressing Enter key submits login form</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>AU-LOGIN18</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>LOGIN_TC_018</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Verify pressing Enter key submits login form</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Open the login page
-Enter username haklarr
-Enter password Icstunnel1
-Press the Enter key on the keyboard</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>Login form is submitted and the user is authenticated successfully.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>AUT-LOGIN19: Verify multiple rapid clicks on login button</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>AU-LOGIN19</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>LOGIN_TC_019</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Verify multiple rapid clicks on login button</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Open the login page
-Enter username haklarr
-Enter password Icstunnel1
-Click the Login button multiple times rapidly</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>System processes the login request safely and does not create duplicate sessions or UI errors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>AUT-LOGIN20: Verify login error message appears after failed login</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>AU-LOGIN20</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>LOGIN_TC_020</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Verify login error message appears after failed login</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Open the login page
-Enter username invaliduser
-Enter password invalidpass
-Click the Login button</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>A visible error message is displayed indicating login failure.</t>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Open browser
+Navigate to http://172.21.166.115/washtabui/login?data=undefined</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Login page loads without errors and displays the login form.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Committing Generated Files 38
</commit_message>
<xml_diff>
--- a/manual_tests/login_approved_manual_tests.xlsx
+++ b/manual_tests/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify login page loads with correct URL and login form</t>
+          <t>Verify login page loads with all required controls</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -488,12 +488,12 @@
         <is>
           <t>Open browser
 Navigate to http://172.21.166.115/washtabui/login?data=undefined
-Wait for the page to fully load</t>
+Observe the login page UI</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Browser URL is http://172.21.166.115/washtabui/login?data=undefined and the login form containing User Name field, Password field, and SIGN IN button is visible.</t>
+          <t>Login page loads successfully at URL containing /washtabui/login and displays User Name textbox labeled 'User Name', Password field labeled 'Password', SIGN IN button, Home control, and Arrow Back control, all visible and enabled.</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify User Name, Password fields and SIGN IN button are visible and enabled</t>
+          <t>Verify successful login using valid credentials via SIGN IN button</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -522,14 +522,14 @@
       <c r="F3" t="inlineStr">
         <is>
           <t>Open the login page URL
-Locate the User Name field
-Locate the Password field
-Locate the SIGN IN button</t>
+Enter 'haklarr' in the User Name field
+Enter 'Icstunnel1' in the Password field
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>User Name textbox and Password password field are visible and editable, and the SIGN IN button is visible and enabled for interaction.</t>
+          <t>User is authenticated and browser redirects to http://172.21.166.115/washtabui/home where the home page UI is visible and the login page is no longer displayed.</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify Home and Arrow Back controls are visible on login page</t>
+          <t>Verify successful login using Enter key from password field</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -558,12 +558,14 @@
       <c r="F4" t="inlineStr">
         <is>
           <t>Open the login page URL
-Observe the navigation area of the page</t>
+Enter 'haklarr' in the User Name field
+Enter 'Icstunnel1' in the Password field
+Press Enter while cursor is in the Password field</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Home control and Arrow Back control are visible and clickable on the login page.</t>
+          <t>Authentication request is submitted and user is redirected to http://172.21.166.115/washtabui/home with the home page UI visible indicating an authenticated session.</t>
         </is>
       </c>
     </row>
@@ -575,12 +577,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Successful login with valid credentials using SIGN IN button</t>
+          <t>Verify login fails with incorrect password</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -592,14 +594,14 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter haklarr in the User Name field
-Enter Icstunnel1 in the Password field
-Click the SIGN IN button</t>
+Enter 'haklarr' in the User Name field
+Enter 'wrongpassword' in the Password field
+Click SIGN IN</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>User is authenticated and redirected to http://172.21.166.115/washtabui/home and the home page is displayed indicating a logged-in state.</t>
+          <t>Authentication is rejected, browser remains on URL containing /washtabui/login, login form stays visible, and a visible authentication failure message indicating invalid username or password is displayed.</t>
         </is>
       </c>
     </row>
@@ -611,12 +613,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Successful login using Enter key from Password field</t>
+          <t>Verify login fails with incorrect username</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -628,14 +630,14 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter haklarr in the User Name field
-Enter Icstunnel1 in the Password field
-Press Enter while cursor focus is in the Password field</t>
+Enter 'invaliduser' in the User Name field
+Enter 'Icstunnel1' in the Password field
+Click SIGN IN</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Login is submitted and the user is authenticated and redirected to http://172.21.166.115/washtabui/home with the home page visible.</t>
+          <t>Authentication is rejected, user remains on the login page at URL containing /washtabui/login, and a visible invalid credentials message is displayed.</t>
         </is>
       </c>
     </row>
@@ -647,7 +649,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Login fails with incorrect password</t>
+          <t>Verify login fails when both username and password are blank</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -664,14 +666,14 @@
       <c r="F7" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter haklarr in the User Name field
-Enter WrongPassword123 in the Password field
-Click the SIGN IN button</t>
+Leave User Name field empty
+Leave Password field empty
+Click SIGN IN</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Authentication fails, browser remains on the login page URL, and a visible login failure message is displayed indicating invalid credentials.</t>
+          <t>Form submission is rejected, browser remains on the login page, and visible required-field validation messages appear for both User Name and Password fields.</t>
         </is>
       </c>
     </row>
@@ -683,7 +685,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Login fails with incorrect username</t>
+          <t>Verify login fails when username is blank</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -700,14 +702,14 @@
       <c r="F8" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter invaliduser in the User Name field
-Enter Icstunnel1 in the Password field
-Click the SIGN IN button</t>
+Leave User Name field empty
+Enter 'Icstunnel1' in Password field
+Click SIGN IN</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Authentication fails, the login page remains displayed, and an error message indicating invalid username or password is visible.</t>
+          <t>Login request is not processed, page remains at URL containing /washtabui/login, and a required-field validation message is displayed for the User Name field.</t>
         </is>
       </c>
     </row>
@@ -719,7 +721,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Validation when both username and password fields are blank</t>
+          <t>Verify login fails when password is blank</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -736,14 +738,14 @@
       <c r="F9" t="inlineStr">
         <is>
           <t>Open the login page URL
-Leave the User Name field empty
-Leave the Password field empty
-Click the SIGN IN button</t>
+Enter 'haklarr' in User Name field
+Leave Password field empty
+Click SIGN IN</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Login is not processed and visible required-field validation messages appear for User Name and Password while remaining on the login page.</t>
+          <t>Login submission is blocked, user remains on the login page, and a required-field validation message is displayed for the Password field.</t>
         </is>
       </c>
     </row>
@@ -755,12 +757,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Validation when username is blank and password is entered</t>
+          <t>Verify Home control navigates to home page</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -772,14 +774,12 @@
       <c r="F10" t="inlineStr">
         <is>
           <t>Open the login page URL
-Leave the User Name field blank
-Enter Icstunnel1 in the Password field
-Click the SIGN IN button</t>
+Click the Home control on the page</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Form submission is blocked and a visible validation message indicates User Name is required while the page remains on the login screen.</t>
+          <t>Browser navigates to http://172.21.166.115/washtabui/home and the home page UI is displayed with URL containing /washtabui/home.</t>
         </is>
       </c>
     </row>
@@ -791,12 +791,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Validation when password is blank and username is entered</t>
+          <t>Verify Arrow Back control navigates to home page</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -808,14 +808,12 @@
       <c r="F11" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter haklarr in the User Name field
-Leave the Password field blank
-Click the SIGN IN button</t>
+Click the Arrow Back control</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Form submission is blocked and a visible validation message indicates Password is required while the login page remains displayed.</t>
+          <t>User is redirected to http://172.21.166.115/washtabui/home and the home page interface is visible with URL containing /washtabui/home.</t>
         </is>
       </c>
     </row>
@@ -827,12 +825,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Login attempt using whitespace-only values</t>
+          <t>Verify password field masks entered characters</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -844,14 +842,13 @@
       <c r="F12" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter spaces only in the User Name field
-Enter spaces only in the Password field
-Click the SIGN IN button</t>
+Enter text into the Password field
+Observe the displayed characters</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Whitespace-only values are treated as invalid input and the login is rejected with validation or authentication error while the login page remains displayed.</t>
+          <t>Characters typed into the Password field are displayed as masked symbols such as dots or asterisks and the actual text value is not visible on screen.</t>
         </is>
       </c>
     </row>
@@ -863,12 +860,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Login with leading and trailing spaces around username</t>
+          <t>Verify login fails when username contains only whitespace</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -880,14 +877,14 @@
       <c r="F13" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter space haklarr space in the User Name field
-Enter Icstunnel1 in the Password field
-Click the SIGN IN button</t>
+Enter only space characters in the User Name field
+Enter 'Icstunnel1' in the Password field
+Click SIGN IN</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Leading and trailing spaces are trimmed before authentication and the user is successfully logged in and redirected to http://172.21.166.115/washtabui/home.</t>
+          <t>Whitespace-only username input is treated as invalid, authentication is rejected, user remains on the login page, and a validation or authentication failure message is displayed.</t>
         </is>
       </c>
     </row>
@@ -899,12 +896,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify password field masks entered characters</t>
+          <t>Verify login fails when password contains only whitespace</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -916,13 +913,14 @@
       <c r="F14" t="inlineStr">
         <is>
           <t>Open the login page URL
-Click inside the Password field
-Type Icstunnel1</t>
+Enter 'haklarr' in User Name field
+Enter only space characters in the Password field
+Click SIGN IN</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Typed characters are displayed as masked symbols such as dots or asterisks and the actual password text is not visible.</t>
+          <t>Whitespace-only password input is rejected, login does not proceed, the login page remains visible, and a validation or authentication failure message is displayed.</t>
         </is>
       </c>
     </row>
@@ -934,12 +932,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Login fails when password case is incorrect</t>
+          <t>Verify login trims leading and trailing spaces in username</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -951,14 +949,14 @@
       <c r="F15" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter haklarr in the User Name field
-Enter icstunnel1 in the Password field
-Click the SIGN IN button</t>
+Enter '  haklarr  ' in the User Name field including leading and trailing spaces
+Enter 'Icstunnel1' in Password field
+Click SIGN IN</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Authentication fails due to incorrect password case, the user remains on the login page, and an invalid credentials error message is visible.</t>
+          <t>System trims leading and trailing whitespace from the username, authenticates successfully, and redirects the user to http://172.21.166.115/washtabui/home with the home page UI visible.</t>
         </is>
       </c>
     </row>
@@ -970,7 +968,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Login fails when username case differs</t>
+          <t>Verify login with extremely long username input</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -987,14 +985,14 @@
       <c r="F16" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter HAKLARR in the User Name field
-Enter Icstunnel1 in the Password field
-Click the SIGN IN button</t>
+Enter a username string longer than 256 characters into the User Name field
+Enter 'Icstunnel1' in Password field
+Click SIGN IN</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Authentication is rejected and the login page remains visible with an invalid credentials error message displayed.</t>
+          <t>System rejects the login attempt or prevents submission, browser remains on URL containing /washtabui/login, a validation or authentication failure message is displayed, and the UI layout remains stable without page errors.</t>
         </is>
       </c>
     </row>
@@ -1006,12 +1004,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Verify Home control redirects to home page</t>
+          <t>Verify multiple rapid clicks on SIGN IN button</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1023,12 +1021,14 @@
       <c r="F17" t="inlineStr">
         <is>
           <t>Open the login page URL
-Click the Home control</t>
+Enter valid username 'haklarr'
+Enter valid password 'Icstunnel1'
+Click the SIGN IN button repeatedly several times in quick succession</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Browser navigates to http://172.21.166.115/washtabui/home and the home page is displayed.</t>
+          <t>Only one authentication request is processed and the browser redirects a single time to http://172.21.166.115/washtabui/home with no duplicate navigation, error messages, or UI instability.</t>
         </is>
       </c>
     </row>
@@ -1040,12 +1040,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Verify Arrow Back control redirects to home page</t>
+          <t>Verify login fails with special characters in username</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1057,156 +1057,14 @@
       <c r="F18" t="inlineStr">
         <is>
           <t>Open the login page URL
-Click the Arrow Back control</t>
+Enter '@@@###$$$' in the User Name field
+Enter 'Icstunnel1' in the Password field
+Click SIGN IN</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Browser navigates to http://172.21.166.115/washtabui/home and the home page loads successfully.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>WT-LOGIN18</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Verify handling of extremely long username input</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Open the login page URL
-Enter a username longer than 256 characters in the User Name field
-Enter Icstunnel1 in the Password field
-Click the SIGN IN button</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Application does not crash and the login attempt fails with an authentication or validation error while the login page remains visible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>WT-LOGIN19</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Login attempt with special characters in username</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Open the login page URL
-Enter haklarr!@# in the User Name field
-Enter Icstunnel1 in the Password field
-Click the SIGN IN button</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Authentication fails, the user remains on the login page, and an invalid credentials or validation error message is displayed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>WT-LOGIN20</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Verify multiple rapid clicks on SIGN IN button do not create duplicate submissions</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Open the login page URL
-Enter haklarr in the User Name field
-Enter Icstunnel1 in the Password field
-Rapidly click the SIGN IN button multiple times</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Only one authentication request is processed and the user is redirected a single time to http://172.21.166.115/washtabui/home without duplicate page loads or errors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>WT-LOGIN21</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Successful login using copied and pasted credentials</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Open the login page URL
-Copy haklarr and paste it into the User Name field
-Copy Icstunnel1 and paste it into the Password field
-Click the SIGN IN button</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Credentials pasted into the fields are accepted and the user is authenticated and redirected to http://172.21.166.115/washtabui/home.</t>
+          <t>Authentication fails, browser remains on the login page at URL containing /washtabui/login, and a visible invalid credentials or validation message is displayed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Committing Generated Files 39
</commit_message>
<xml_diff>
--- a/manual_tests/login_approved_manual_tests.xlsx
+++ b/manual_tests/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify login page loads with all required controls</t>
+          <t>Verify login page loads and UI elements are visible</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,14 +486,19 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Open browser
-Navigate to http://172.21.166.115/washtabui/login?data=undefined
-Observe the login page UI</t>
+          <t>Open the login page URL http://172.21.166.115/washtabui/login?data=undefined
+Observe the login page interface
+Verify User Name textbox is visible
+Verify Password field is visible
+Verify characters entered into Password field are masked
+Verify SIGN IN button is visible
+Verify Home control is visible
+Verify Arrow Back control is visible</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Login page loads successfully at URL containing /washtabui/login and displays User Name textbox labeled 'User Name', Password field labeled 'Password', SIGN IN button, Home control, and Arrow Back control, all visible and enabled.</t>
+          <t>Login page loads without error and displays User Name textbox, Password masked input field, SIGN IN button, Home control, and Arrow Back control. The browser URL remains http://172.21.166.115/washtabui/login?data=undefined.</t>
         </is>
       </c>
     </row>
@@ -505,7 +510,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify successful login using valid credentials via SIGN IN button</t>
+          <t>Successful login using valid credentials with SIGN IN button</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -522,14 +527,14 @@
       <c r="F3" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter 'haklarr' in the User Name field
-Enter 'Icstunnel1' in the Password field
+Enter haklarr in the User Name field
+Enter Icstunnel1 in the Password field
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>User is authenticated and browser redirects to http://172.21.166.115/washtabui/home where the home page UI is visible and the login page is no longer displayed.</t>
+          <t>User authentication succeeds and browser navigates to http://172.21.166.115/washtabui/home. The home page content is displayed and the login page is no longer visible.</t>
         </is>
       </c>
     </row>
@@ -541,7 +546,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify successful login using Enter key from password field</t>
+          <t>Successful login using Enter key from password field</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -558,14 +563,14 @@
       <c r="F4" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter 'haklarr' in the User Name field
-Enter 'Icstunnel1' in the Password field
-Press Enter while cursor is in the Password field</t>
+Enter haklarr in the User Name field
+Enter Icstunnel1 in the Password field
+Press Enter while focus is inside the Password field</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Authentication request is submitted and user is redirected to http://172.21.166.115/washtabui/home with the home page UI visible indicating an authenticated session.</t>
+          <t>User authentication succeeds and the browser redirects to http://172.21.166.115/washtabui/home with the home page interface visible.</t>
         </is>
       </c>
     </row>
@@ -577,7 +582,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify login fails with incorrect password</t>
+          <t>Login fails with incorrect password</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -594,14 +599,14 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter 'haklarr' in the User Name field
-Enter 'wrongpassword' in the Password field
-Click SIGN IN</t>
+Enter haklarr in the User Name field
+Enter WrongPassword123 in the Password field
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Authentication is rejected, browser remains on URL containing /washtabui/login, login form stays visible, and a visible authentication failure message indicating invalid username or password is displayed.</t>
+          <t>Authentication is rejected. A visible login failure message indicating incorrect username or password appears and the browser remains on the login page URL.</t>
         </is>
       </c>
     </row>
@@ -613,7 +618,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify login fails with incorrect username</t>
+          <t>Login fails with incorrect username</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -630,14 +635,14 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter 'invaliduser' in the User Name field
-Enter 'Icstunnel1' in the Password field
-Click SIGN IN</t>
+Enter wronguser in the User Name field
+Enter Icstunnel1 in the Password field
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Authentication is rejected, user remains on the login page at URL containing /washtabui/login, and a visible invalid credentials message is displayed.</t>
+          <t>Authentication fails and an observable error message indicating invalid username or password is displayed while the browser remains on the login page.</t>
         </is>
       </c>
     </row>
@@ -649,7 +654,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify login fails when both username and password are blank</t>
+          <t>Login fails when both username and password are blank</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -668,12 +673,12 @@
           <t>Open the login page URL
 Leave User Name field empty
 Leave Password field empty
-Click SIGN IN</t>
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Form submission is rejected, browser remains on the login page, and visible required-field validation messages appear for both User Name and Password fields.</t>
+          <t>Login is blocked. Required field validation indicators appear for both User Name and Password fields and the browser remains on the login page.</t>
         </is>
       </c>
     </row>
@@ -685,7 +690,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify login fails when username is blank</t>
+          <t>Login fails when username is blank</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -703,13 +708,13 @@
         <is>
           <t>Open the login page URL
 Leave User Name field empty
-Enter 'Icstunnel1' in Password field
-Click SIGN IN</t>
+Enter Icstunnel1 in the Password field
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Login request is not processed, page remains at URL containing /washtabui/login, and a required-field validation message is displayed for the User Name field.</t>
+          <t>Submission is rejected with a visible validation message indicating User Name is required and the page remains on the login screen.</t>
         </is>
       </c>
     </row>
@@ -721,7 +726,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify login fails when password is blank</t>
+          <t>Login fails when password is blank</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -738,14 +743,14 @@
       <c r="F9" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter 'haklarr' in User Name field
+Enter haklarr in the User Name field
 Leave Password field empty
-Click SIGN IN</t>
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Login submission is blocked, user remains on the login page, and a required-field validation message is displayed for the Password field.</t>
+          <t>Submission is rejected with a visible validation message indicating Password is required and the login page remains displayed.</t>
         </is>
       </c>
     </row>
@@ -757,7 +762,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify Home control navigates to home page</t>
+          <t>Password field masks entered characters</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -774,12 +779,13 @@
       <c r="F10" t="inlineStr">
         <is>
           <t>Open the login page URL
-Click the Home control on the page</t>
+Click inside the Password field
+Type Icstunnel1</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Browser navigates to http://172.21.166.115/washtabui/home and the home page UI is displayed with URL containing /washtabui/home.</t>
+          <t>Each typed character in the Password field appears as a masked symbol such as dots or asterisks instead of displaying the actual characters.</t>
         </is>
       </c>
     </row>
@@ -791,7 +797,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify Arrow Back control navigates to home page</t>
+          <t>Navigation using Home control from login page</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -808,12 +814,12 @@
       <c r="F11" t="inlineStr">
         <is>
           <t>Open the login page URL
-Click the Arrow Back control</t>
+Click the Home control</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>User is redirected to http://172.21.166.115/washtabui/home and the home page interface is visible with URL containing /washtabui/home.</t>
+          <t>Browser navigates to http://172.21.166.115/washtabui/home and the home page UI becomes visible.</t>
         </is>
       </c>
     </row>
@@ -825,7 +831,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify password field masks entered characters</t>
+          <t>Navigation using Arrow Back control from login page</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -842,13 +848,12 @@
       <c r="F12" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter text into the Password field
-Observe the displayed characters</t>
+Click the Arrow Back control</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Characters typed into the Password field are displayed as masked symbols such as dots or asterisks and the actual text value is not visible on screen.</t>
+          <t>Browser redirects to http://172.21.166.115/washtabui/home and the home page content loads successfully.</t>
         </is>
       </c>
     </row>
@@ -860,12 +865,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify login fails when username contains only whitespace</t>
+          <t>Login with leading and trailing spaces in username</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -877,14 +882,14 @@
       <c r="F13" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter only space characters in the User Name field
-Enter 'Icstunnel1' in the Password field
-Click SIGN IN</t>
+Enter '  haklarr  ' in the User Name field including leading and trailing spaces
+Enter Icstunnel1 in the Password field
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Whitespace-only username input is treated as invalid, authentication is rejected, user remains on the login page, and a validation or authentication failure message is displayed.</t>
+          <t>System trims leading and trailing spaces from the username before authentication and successfully redirects the user to http://172.21.166.115/washtabui/home.</t>
         </is>
       </c>
     </row>
@@ -896,7 +901,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify login fails when password contains only whitespace</t>
+          <t>Login attempt with whitespace-only username</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -913,14 +918,14 @@
       <c r="F14" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter 'haklarr' in User Name field
-Enter only space characters in the Password field
-Click SIGN IN</t>
+Enter multiple spaces in the User Name field
+Enter Icstunnel1 in the Password field
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Whitespace-only password input is rejected, login does not proceed, the login page remains visible, and a validation or authentication failure message is displayed.</t>
+          <t>System treats the username as empty and displays a required-field validation for User Name while remaining on the login page.</t>
         </is>
       </c>
     </row>
@@ -932,12 +937,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify login trims leading and trailing spaces in username</t>
+          <t>Login attempt with whitespace-only password</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -949,14 +954,14 @@
       <c r="F15" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter '  haklarr  ' in the User Name field including leading and trailing spaces
-Enter 'Icstunnel1' in Password field
-Click SIGN IN</t>
+Enter haklarr in the User Name field
+Enter multiple spaces in the Password field
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>System trims leading and trailing whitespace from the username, authenticates successfully, and redirects the user to http://172.21.166.115/washtabui/home with the home page UI visible.</t>
+          <t>Authentication is rejected and a validation or login failure message appears while the browser remains on the login page.</t>
         </is>
       </c>
     </row>
@@ -968,7 +973,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify login with extremely long username input</t>
+          <t>Login attempt with excessively long username input</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -985,14 +990,14 @@
       <c r="F16" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter a username string longer than 256 characters into the User Name field
-Enter 'Icstunnel1' in Password field
-Click SIGN IN</t>
+Enter a username string longer than 200 characters in the User Name field
+Enter Icstunnel1 in the Password field
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>System rejects the login attempt or prevents submission, browser remains on URL containing /washtabui/login, a validation or authentication failure message is displayed, and the UI layout remains stable without page errors.</t>
+          <t>Application does not crash or break UI layout. Authentication fails and an error message is shown while the user remains on the login page.</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1009,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Verify multiple rapid clicks on SIGN IN button</t>
+          <t>Login attempt with special characters in username</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1021,14 +1026,14 @@
       <c r="F17" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter valid username 'haklarr'
-Enter valid password 'Icstunnel1'
-Click the SIGN IN button repeatedly several times in quick succession</t>
+Enter user!@# in the User Name field
+Enter Icstunnel1 in the Password field
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Only one authentication request is processed and the browser redirects a single time to http://172.21.166.115/washtabui/home with no duplicate navigation, error messages, or UI instability.</t>
+          <t>Authentication fails and a visible login error message appears while the page remains on the login screen.</t>
         </is>
       </c>
     </row>
@@ -1040,12 +1045,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Verify login fails with special characters in username</t>
+          <t>Repeated clicking of SIGN IN button during login attempt</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1057,14 +1062,50 @@
       <c r="F18" t="inlineStr">
         <is>
           <t>Open the login page URL
-Enter '@@@###$$$' in the User Name field
-Enter 'Icstunnel1' in the Password field
-Click SIGN IN</t>
+Enter haklarr in the User Name field
+Enter Icstunnel1 in the Password field
+Rapidly click the SIGN IN button multiple times</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Authentication fails, browser remains on the login page at URL containing /washtabui/login, and a visible invalid credentials or validation message is displayed.</t>
+          <t>Only one authentication process is executed and the browser performs a single redirect to http://172.21.166.115/washtabui/home without duplicate navigation or UI errors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>WT-LOGIN18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Login attempt with correct username but wrong case password</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Open the login page URL
+Enter haklarr in the User Name field
+Enter icstunnel1 in the Password field
+Click the SIGN IN button</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Authentication fails due to password case sensitivity. An invalid credential message appears and the browser remains on the login page.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Committing Generated Files 41
</commit_message>
<xml_diff>
--- a/manual_tests/login_approved_manual_tests.xlsx
+++ b/manual_tests/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify login page UI elements are visible</t>
+          <t>Verify login page loads with correct URL and login form is visible</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,18 +486,13 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Navigate to http://172.21.166.115/washtabui/login?data=undefined
-Verify the browser URL matches the login page URL
-Check presence of username_textbox
-Check presence of password_textbox
-Check presence of sign_in_button
-Check presence of back_navigation_button
-Check presence of home_navigation_button</t>
+          <t>Open a browser
+Navigate to http://172.21.166.115/washtabui/login?data=undefined</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Login page loads successfully at the specified URL and the username_textbox, password_textbox, SIGN IN button, back_navigation_button, and home_navigation_button are visible and interactable.</t>
+          <t>Login page loads successfully, the browser URL is http://172.21.166.115/washtabui/login?data=undefined, and the username textbox, password textbox, SIGN IN button, back navigation button, and home navigation button are visible</t>
         </is>
       </c>
     </row>
@@ -509,7 +504,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Login with valid username and password</t>
+          <t>Verify username textbox accepts input</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -525,15 +520,14 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Navigate to the login page URL
-Enter hacklarr in username_textbox
-Enter Icstunnel1 in password_textbox
-Click sign_in_button</t>
+          <t>Navigate to the login page
+Click on the username textbox
+Enter hacklarr into the username textbox</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>User authentication succeeds and the application redirects to http://172.21.166.115/washtabui/home with the home page fully loaded and the login page no longer visible.</t>
+          <t>Entered text hacklarr is displayed in the username textbox and the field remains editable</t>
         </is>
       </c>
     </row>
@@ -545,12 +539,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Login with invalid username and valid password</t>
+          <t>Verify password textbox masks entered characters</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -561,15 +555,14 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Navigate to the login page URL
-Enter invaliduser in username_textbox
-Enter Icstunnel1 in password_textbox
-Click sign_in_button</t>
+          <t>Navigate to the login page
+Click the password textbox
+Enter Icstunnel1 into the password textbox</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Authentication fails, the user remains on the login page, the browser URL does not change to the home page URL, and a visible login failure message such as 'Sign in failed' or equivalent authentication error is displayed.</t>
+          <t>Password characters are masked (for example shown as dots or asterisks) and the actual password text is not visible on the screen</t>
         </is>
       </c>
     </row>
@@ -581,12 +574,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Login with valid username and invalid password</t>
+          <t>Verify successful login with valid credentials</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -597,15 +590,15 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Navigate to the login page URL
-Enter hacklarr in username_textbox
-Enter wrongpassword in password_textbox
-Click sign_in_button</t>
+          <t>Navigate to the login page
+Enter hacklarr into the username textbox
+Enter Icstunnel1 into the password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Authentication fails, the login page remains displayed, the URL does not change to the home page URL, and a visible authentication failure message is shown.</t>
+          <t>User authentication succeeds and the application redirects to the home page with URL http://172.21.166.115/washtabui/home and the login page is no longer displayed</t>
         </is>
       </c>
     </row>
@@ -617,7 +610,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Attempt login with empty username and password</t>
+          <t>Verify login fails with invalid username and valid password</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -633,15 +626,15 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Navigate to the login page URL
-Leave username_textbox empty
-Leave password_textbox empty
-Click sign_in_button</t>
+          <t>Navigate to the login page
+Enter invaliduser into the username textbox
+Enter Icstunnel1 into the password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Login is rejected, the user remains on the login page, the home page URL is not loaded, and the form displays a validation or authentication error preventing login.</t>
+          <t>Authentication fails, an error message indicating invalid or incorrect credentials is displayed, and the browser remains on the login page URL</t>
         </is>
       </c>
     </row>
@@ -653,7 +646,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Attempt login with valid username and empty password</t>
+          <t>Verify login fails with valid username and invalid password</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -669,15 +662,15 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Navigate to the login page URL
-Enter hacklarr in username_textbox
-Leave password_textbox empty
-Click sign_in_button</t>
+          <t>Navigate to the login page
+Enter hacklarr into the username textbox
+Enter wrongpassword into the password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Authentication fails, the application remains on the login page without redirecting to the home page URL, and a visible validation or login error is displayed.</t>
+          <t>Authentication fails, an invalid or incorrect credentials message is displayed, and the login page remains visible without redirecting to the home page</t>
         </is>
       </c>
     </row>
@@ -689,12 +682,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify password field masks entered characters</t>
+          <t>Verify login fails when both username and password are invalid</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -705,15 +698,15 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Navigate to the login page URL
-Click password_textbox
-Enter Icstunnel1 in password_textbox
-Observe how characters are displayed</t>
+          <t>Navigate to the login page
+Enter invaliduser into the username textbox
+Enter invalidpassword into the password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Characters entered into password_textbox are displayed as masked symbols (such as dots or asterisks) and the actual password text is not visible on screen.</t>
+          <t>Authentication fails, an invalid credentials error message is displayed, and the application remains on the login page</t>
         </is>
       </c>
     </row>
@@ -725,12 +718,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify back navigation button redirects to home page</t>
+          <t>Verify login fails when username and password fields are empty</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -741,13 +734,15 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Navigate to the login page URL
-Click back_navigation_button</t>
+          <t>Navigate to the login page
+Leave username textbox empty
+Leave password textbox empty
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Application navigates away from the login page and loads the home page with the browser URL changing to http://172.21.166.115/washtabui/home.</t>
+          <t>Login attempt is rejected, the user remains on the login page, and an authentication or validation message indicating invalid or missing credentials is displayed</t>
         </is>
       </c>
     </row>
@@ -759,12 +754,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify home navigation button redirects to home page</t>
+          <t>Verify login fails when username is empty and password is provided</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -775,13 +770,15 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Navigate to the login page URL
-Click home_navigation_button</t>
+          <t>Navigate to the login page
+Leave username textbox empty
+Enter Icstunnel1 into the password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Application redirects to the home page and the browser URL becomes http://172.21.166.115/washtabui/home with the login page no longer displayed.</t>
+          <t>Login attempt fails, an error or validation message is displayed, and the application remains on the login page without redirecting</t>
         </is>
       </c>
     </row>
@@ -793,12 +790,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Login attempt with leading and trailing whitespace in username</t>
+          <t>Verify login fails when password is empty and username is provided</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -809,15 +806,15 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Navigate to the login page URL
-Enter '  hacklarr  ' in username_textbox including spaces before and after the username
-Enter Icstunnel1 in password_textbox
-Click sign_in_button</t>
+          <t>Navigate to the login page
+Enter hacklarr into the username textbox
+Leave password textbox empty
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>System processes the entered value and rejects authentication, the user remains on the login page, the URL does not change to the home page URL, and a login failure message is displayed.</t>
+          <t>Authentication fails, an error or validation message is displayed, and the user stays on the login page without navigation to the home page</t>
         </is>
       </c>
     </row>
@@ -829,12 +826,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Login with very long username value</t>
+          <t>Verify back navigation button redirects user to home page</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -845,15 +842,13 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Navigate to the login page URL
-Enter a username string significantly longer than a typical username length in username_textbox
-Enter Icstunnel1 in password_textbox
-Click sign_in_button</t>
+          <t>Navigate to the login page
+Click the back navigation button</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Application safely rejects the authentication attempt, the login page remains displayed, no navigation to the home page occurs, and the UI remains stable without page crash or layout break.</t>
+          <t>Application navigates away from the login page and loads the home page with URL http://172.21.166.115/washtabui/home</t>
         </is>
       </c>
     </row>
@@ -865,12 +860,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Login with special characters in username</t>
+          <t>Verify home navigation button redirects user to home page</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -881,15 +876,13 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Navigate to the login page URL
-Enter user!@# in username_textbox
-Enter Icstunnel1 in password_textbox
-Click sign_in_button</t>
+          <t>Navigate to the login page
+Click the home navigation button</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Authentication fails, the user stays on the login page, the home page URL is not loaded, and an authentication failure message is displayed.</t>
+          <t>User is redirected to the home page and the browser URL changes to http://172.21.166.115/washtabui/home</t>
         </is>
       </c>
     </row>
@@ -901,7 +894,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Rapid multiple clicks on SIGN IN button with valid credentials</t>
+          <t>Verify login behavior with leading and trailing spaces in credentials</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -917,15 +910,195 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Navigate to the login page URL
-Enter hacklarr in username_textbox
-Enter Icstunnel1 in password_textbox
-Rapidly click sign_in_button multiple times</t>
+          <t>Navigate to the login page
+Enter '  hacklarr  ' into the username textbox
+Enter '  Icstunnel1  ' into the password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>System processes only one authentication request and redirects a single time to http://172.21.166.115/washtabui/home without duplicate navigation, duplicate sessions, or UI errors.</t>
+          <t>Application processes the entered credentials and either trims whitespace and logs the user in successfully to the home page URL http://172.21.166.115/washtabui/home or rejects the login with an invalid credentials message while remaining on the login page</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>WT-LOGIN14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Verify login fails with extremely long username and password values</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Navigate to the login page
+Enter a username longer than 200 characters into the username textbox
+Enter a password longer than 200 characters into the password textbox
+Click the SIGN IN button</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Login attempt is rejected, the application remains on the login page, and the UI remains stable without page crash, layout break, or unexpected redirect</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>WT-LOGIN15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Verify system handles multiple rapid clicks on SIGN IN button</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Navigate to the login page
+Enter hacklarr into the username textbox
+Enter Icstunnel1 into the password textbox
+Rapidly click the SIGN IN button multiple times</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Only a single authentication request is processed and the user is redirected once to the home page without duplicate navigation or visible application errors</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>WT-LOGIN16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Verify login fails when username and password contain only whitespace</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Navigate to the login page
+Enter only spaces into the username textbox
+Enter only spaces into the password textbox
+Click the SIGN IN button</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Login attempt is rejected, an authentication or validation error message is displayed, and the application remains on the login page</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>WT-LOGIN17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Verify login submission using Enter key with valid credentials</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Navigate to the login page
+Enter hacklarr into the username textbox
+Enter Icstunnel1 into the password textbox
+Press the Enter key on the keyboard</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Login form is submitted and the user is successfully authenticated and redirected to the home page with URL http://172.21.166.115/washtabui/home</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>WT-LOGIN18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Verify login fails with special characters in username and password</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Navigate to the login page
+Enter !@#$$% into the username textbox
+Enter !@#$$% into the password textbox
+Click the SIGN IN button</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Authentication fails, an invalid or incorrect credentials message is displayed, and the browser remains on the login page without redirecting to the home page</t>
         </is>
       </c>
     </row>

</xml_diff>